<commit_message>
update user account import
</commit_message>
<xml_diff>
--- a/src/src/main/webapp/portal/uaa/userAccount/APM_UserAccount_Template.xlsx
+++ b/src/src/main/webapp/portal/uaa/userAccount/APM_UserAccount_Template.xlsx
@@ -14,10 +14,10 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="34">
   <si>
-    <t>所属集团</t>
+    <t>所属集团*</t>
   </si>
   <si>
-    <t>所属医院*</t>
+    <t>所属医院</t>
   </si>
   <si>
     <t>所属院区</t>
@@ -394,31 +394,31 @@
     <xf numFmtId="49" fontId="3" fillId="2" borderId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" borderId="11" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="11" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="0" borderId="1" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="12" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="4" borderId="13" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="4" fillId="3" borderId="13" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="0" borderId="14" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="14" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="4" borderId="15" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="15" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
     <xf numFmtId="49" fontId="3" fillId="2" borderId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" borderId="11" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="11" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="4" borderId="14" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="14" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
   </cellXfs>
@@ -3881,7 +3881,7 @@
     <col min="6" max="256" width="8.85156" style="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="13.65" customHeight="1">
+    <row r="1" ht="13.7" customHeight="1">
       <c r="A1" t="s" s="13">
         <v>15</v>
       </c>
@@ -3890,14 +3890,14 @@
       <c r="D1" s="15"/>
       <c r="E1" s="15"/>
     </row>
-    <row r="2" ht="13.65" customHeight="1">
+    <row r="2" ht="13.7" customHeight="1">
       <c r="A2" s="16"/>
       <c r="B2" s="14"/>
       <c r="C2" s="15"/>
       <c r="D2" s="15"/>
       <c r="E2" s="15"/>
     </row>
-    <row r="3" ht="16" customHeight="1">
+    <row r="3" ht="15.95" customHeight="1">
       <c r="A3" t="s" s="17">
         <v>16</v>
       </c>
@@ -3906,7 +3906,7 @@
       <c r="D3" s="15"/>
       <c r="E3" s="15"/>
     </row>
-    <row r="4" ht="16" customHeight="1">
+    <row r="4" ht="15.95" customHeight="1">
       <c r="A4" t="s" s="17">
         <v>17</v>
       </c>
@@ -3915,7 +3915,7 @@
       <c r="D4" s="15"/>
       <c r="E4" s="15"/>
     </row>
-    <row r="5" ht="16" customHeight="1">
+    <row r="5" ht="15.95" customHeight="1">
       <c r="A5" t="s" s="17">
         <v>18</v>
       </c>
@@ -3924,7 +3924,7 @@
       <c r="D5" s="15"/>
       <c r="E5" s="15"/>
     </row>
-    <row r="6" ht="16" customHeight="1">
+    <row r="6" ht="15.95" customHeight="1">
       <c r="A6" t="s" s="17">
         <v>19</v>
       </c>
@@ -3933,7 +3933,7 @@
       <c r="D6" s="15"/>
       <c r="E6" s="15"/>
     </row>
-    <row r="7" ht="16" customHeight="1">
+    <row r="7" ht="15.95" customHeight="1">
       <c r="A7" t="s" s="17">
         <v>20</v>
       </c>
@@ -3942,7 +3942,7 @@
       <c r="D7" s="15"/>
       <c r="E7" s="15"/>
     </row>
-    <row r="8" ht="16" customHeight="1">
+    <row r="8" ht="15.95" customHeight="1">
       <c r="A8" t="s" s="17">
         <v>21</v>
       </c>
@@ -3951,7 +3951,7 @@
       <c r="D8" s="15"/>
       <c r="E8" s="15"/>
     </row>
-    <row r="9" ht="16" customHeight="1">
+    <row r="9" ht="15.95" customHeight="1">
       <c r="A9" t="s" s="17">
         <v>22</v>
       </c>
@@ -3960,14 +3960,14 @@
       <c r="D9" s="15"/>
       <c r="E9" s="15"/>
     </row>
-    <row r="10" ht="16" customHeight="1">
+    <row r="10" ht="15.95" customHeight="1">
       <c r="A10" s="19"/>
       <c r="B10" s="14"/>
       <c r="C10" s="15"/>
       <c r="D10" s="15"/>
       <c r="E10" s="15"/>
     </row>
-    <row r="11" ht="13.65" customHeight="1">
+    <row r="11" ht="13.7" customHeight="1">
       <c r="A11" t="s" s="20">
         <v>23</v>
       </c>
@@ -3983,7 +3983,7 @@
       <c r="D12" s="15"/>
       <c r="E12" s="15"/>
     </row>
-    <row r="13" ht="16" customHeight="1">
+    <row r="13" ht="15.95" customHeight="1">
       <c r="A13" t="s" s="17">
         <v>24</v>
       </c>
@@ -3992,7 +3992,7 @@
       <c r="D13" s="15"/>
       <c r="E13" s="15"/>
     </row>
-    <row r="14" ht="16" customHeight="1">
+    <row r="14" ht="15.95" customHeight="1">
       <c r="A14" t="s" s="17">
         <v>25</v>
       </c>
@@ -4001,7 +4001,7 @@
       <c r="D14" s="15"/>
       <c r="E14" s="15"/>
     </row>
-    <row r="15" ht="16" customHeight="1">
+    <row r="15" ht="15.95" customHeight="1">
       <c r="A15" t="s" s="17">
         <v>26</v>
       </c>
@@ -4010,7 +4010,7 @@
       <c r="D15" s="15"/>
       <c r="E15" s="15"/>
     </row>
-    <row r="16" ht="16" customHeight="1">
+    <row r="16" ht="15.95" customHeight="1">
       <c r="A16" t="s" s="17">
         <v>27</v>
       </c>
@@ -4019,7 +4019,7 @@
       <c r="D16" s="15"/>
       <c r="E16" s="15"/>
     </row>
-    <row r="17" ht="16" customHeight="1">
+    <row r="17" ht="15.95" customHeight="1">
       <c r="A17" t="s" s="17">
         <v>28</v>
       </c>
@@ -4028,7 +4028,7 @@
       <c r="D17" s="15"/>
       <c r="E17" s="15"/>
     </row>
-    <row r="18" ht="16" customHeight="1">
+    <row r="18" ht="15.95" customHeight="1">
       <c r="A18" t="s" s="17">
         <v>29</v>
       </c>
@@ -4037,7 +4037,7 @@
       <c r="D18" s="15"/>
       <c r="E18" s="15"/>
     </row>
-    <row r="19" ht="16" customHeight="1">
+    <row r="19" ht="15.95" customHeight="1">
       <c r="A19" t="s" s="17">
         <v>30</v>
       </c>
@@ -4046,7 +4046,7 @@
       <c r="D19" s="15"/>
       <c r="E19" s="15"/>
     </row>
-    <row r="20" ht="16" customHeight="1">
+    <row r="20" ht="15.95" customHeight="1">
       <c r="A20" t="s" s="17">
         <v>31</v>
       </c>
@@ -4055,7 +4055,7 @@
       <c r="D20" s="15"/>
       <c r="E20" s="15"/>
     </row>
-    <row r="21" ht="16" customHeight="1">
+    <row r="21" ht="15.95" customHeight="1">
       <c r="A21" t="s" s="17">
         <v>32</v>
       </c>
@@ -4075,8 +4075,8 @@
     </row>
   </sheetData>
   <mergeCells count="2">
+    <mergeCell ref="A11:A12"/>
     <mergeCell ref="A1:A2"/>
-    <mergeCell ref="A11:A12"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup firstPageNumber="1" fitToHeight="1" fitToWidth="1" scale="100" useFirstPageNumber="0" orientation="portrait" pageOrder="downThenOver"/>

</xml_diff>